<commit_message>
documentacion de cierre sprint 4
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencia del Proyecto/Evidencias de documentacion/Metodologia Scrum/Sprint 01234/Sprint 2/Burndown Sprint2 SOC.xlsx
+++ b/Fase 2/Evidencia del Proyecto/Evidencias de documentacion/Metodologia Scrum/Sprint 01234/Sprint 2/Burndown Sprint2 SOC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\munoz\Desktop\Fase 1\Fase dos\Sptint1,2,3,4\Sprint 2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\munoz\Desktop\Fase 1\Fase 2\Evidencia del Proyecto\Evidencias de documentacion\Metodologia Scrum\Sprint 01234\Sprint 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5EB8AB7A-304C-437A-8166-1F110764F100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22C431EA-C7E0-4282-90BB-B0C766639BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="S2_Burndown" sheetId="3" r:id="rId1"/>
@@ -54,13 +54,13 @@
     <t>Objetivo</t>
   </si>
   <si>
-    <t>Sprint 1</t>
-  </si>
-  <si>
     <t>15</t>
   </si>
   <si>
     <t>Módulo Gestion operacional</t>
+  </si>
+  <si>
+    <t>Sprint 2</t>
   </si>
 </sst>
 </file>
@@ -1093,7 +1093,7 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -1117,7 +1117,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -1125,7 +1125,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>